<commit_message>
received checklist, shipment dropdown, code checks
</commit_message>
<xml_diff>
--- a/Stock_Control/INRIPE_Stock_Entry_v1.xlsx
+++ b/Stock_Control/INRIPE_Stock_Entry_v1.xlsx
@@ -36,12 +36,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="dd\-mmm\-yy\ hh:mm"/>
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
-    <numFmt numFmtId="167" formatCode="dd-mmm-yy"/>
-    <numFmt numFmtId="168" formatCode="dd-mmm-yy hh:mm"/>
+    <numFmt numFmtId="167" formatCode="dd\-mmm\-yy"/>
+    <numFmt numFmtId="168" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="169" formatCode="dd-mmm-yy"/>
   </numFmts>
   <fonts count="23">
     <font>
@@ -361,7 +362,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -477,6 +478,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -489,10 +492,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1022,8 +1022,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="tblShipment" displayName="tblShipment" ref="A6:I22" headerRowCount="1">
-  <autoFilter ref="A6:I22"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="tblShipment" displayName="tblShipment" ref="A6:I24" headerRowCount="1">
+  <autoFilter ref="A6:I24"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Shipment No"/>
     <tableColumn id="2" name="Market"/>
@@ -1271,83 +1271,83 @@
   <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col width="2" customWidth="1" style="52" min="1" max="1"/>
-    <col width="16" customWidth="1" style="52" min="2" max="2"/>
-    <col width="13" customWidth="1" style="52" min="3" max="3"/>
-    <col width="46" customWidth="1" style="52" min="4" max="4"/>
-    <col width="34" customWidth="1" style="52" min="5" max="5"/>
+    <col width="2" customWidth="1" style="54" min="1" max="1"/>
+    <col width="16" customWidth="1" style="54" min="2" max="2"/>
+    <col width="13" customWidth="1" style="54" min="3" max="3"/>
+    <col width="46" customWidth="1" style="54" min="4" max="4"/>
+    <col width="34" customWidth="1" style="54" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="52">
+    <row r="1" ht="25.5" customHeight="1" s="54">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>GUIDE</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="52">
+    <row r="2" ht="15" customHeight="1" s="54">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>One page. Read once.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="27.75" customHeight="1" s="52">
-      <c r="B4" s="50" t="inlineStr">
+    <row r="4" ht="27.75" customHeight="1" s="54">
+      <c r="B4" s="52" t="inlineStr">
         <is>
           <t>GOLDEN RULE:   type only what physically happened.   Stock only ever moves through MOVES.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="52">
+    <row r="6" ht="15" customHeight="1" s="54">
       <c r="B6" s="3" t="n"/>
-      <c r="C6" s="53" t="inlineStr">
+      <c r="C6" s="55" t="inlineStr">
         <is>
           <t>BLUE  =  you type here</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="52">
+    <row r="7" ht="15" customHeight="1" s="54">
       <c r="B7" s="4" t="n"/>
-      <c r="C7" s="53" t="inlineStr">
+      <c r="C7" s="55" t="inlineStr">
         <is>
           <t>GREY  =  the workbook works it out</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="52">
+    <row r="8" ht="15" customHeight="1" s="54">
       <c r="B8" s="5" t="n"/>
-      <c r="C8" s="53" t="inlineStr">
+      <c r="C8" s="55" t="inlineStr">
         <is>
           <t>YELLOW  =  a setting you may change</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="52">
+    <row r="9" ht="15" customHeight="1" s="54">
       <c r="B9" s="6" t="n"/>
-      <c r="C9" s="53" t="inlineStr">
+      <c r="C9" s="55" t="inlineStr">
         <is>
           <t>RED  =  fix this row</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="52">
+    <row r="10" ht="15" customHeight="1" s="54">
       <c r="B10" s="7" t="n"/>
-      <c r="C10" s="53" t="inlineStr">
+      <c r="C10" s="55" t="inlineStr">
         <is>
           <t>GREEN  =  stock coming IN</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="52">
+    <row r="11" ht="15" customHeight="1" s="54">
       <c r="B11" s="8" t="n"/>
-      <c r="C11" s="53" t="inlineStr">
+      <c r="C11" s="55" t="inlineStr">
         <is>
           <t>PINK  =  stock going OUT</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1" s="52">
+    <row r="14" ht="24" customHeight="1" s="54">
       <c r="B14" s="9" t="inlineStr">
         <is>
           <t>Sheet</t>
@@ -1364,211 +1364,211 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1" s="52">
+    <row r="15" ht="15" customHeight="1" s="54">
       <c r="B15" s="10" t="inlineStr">
         <is>
           <t>SHIPMENTS</t>
         </is>
       </c>
-      <c r="C15" s="51" t="inlineStr">
+      <c r="C15" s="53" t="inlineStr">
         <is>
           <t>Per shipment</t>
         </is>
       </c>
-      <c r="D15" s="51" t="inlineStr">
+      <c r="D15" s="53" t="inlineStr">
         <is>
           <t>6 fields: Shipment No, Market, Arrival Date, Source, Item Name, Shipped Qty</t>
         </is>
       </c>
-      <c r="E15" s="54" t="n"/>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="52">
+      <c r="E15" s="56" t="n"/>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="54">
       <c r="B16" s="12" t="inlineStr">
         <is>
           <t>MOVES</t>
         </is>
       </c>
-      <c r="C16" s="49" t="inlineStr">
+      <c r="C16" s="51" t="inlineStr">
         <is>
           <t>Daily</t>
         </is>
       </c>
-      <c r="D16" s="49" t="inlineStr">
+      <c r="D16" s="51" t="inlineStr">
         <is>
           <t>6 fields at most. Pick the Movement and it tells you which ones.</t>
         </is>
       </c>
-      <c r="E16" s="54" t="n"/>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="52">
+      <c r="E16" s="56" t="n"/>
+    </row>
+    <row r="17" ht="15" customHeight="1" s="54">
       <c r="B17" s="10" t="inlineStr">
         <is>
           <t>COUNT</t>
         </is>
       </c>
-      <c r="C17" s="51" t="inlineStr">
+      <c r="C17" s="53" t="inlineStr">
         <is>
           <t>Weekly</t>
         </is>
       </c>
-      <c r="D17" s="51" t="inlineStr">
+      <c r="D17" s="53" t="inlineStr">
         <is>
           <t>4 fields: Date, Shipment No, Item Name, Physical Qty</t>
         </is>
       </c>
-      <c r="E17" s="54" t="n"/>
-    </row>
-    <row r="18" ht="21.75" customHeight="1" s="52">
+      <c r="E17" s="56" t="n"/>
+    </row>
+    <row r="18" ht="21.75" customHeight="1" s="54">
       <c r="B18" s="12" t="inlineStr">
         <is>
           <t>DISPATCH</t>
         </is>
       </c>
-      <c r="C18" s="49" t="inlineStr">
+      <c r="C18" s="51" t="inlineStr">
         <is>
           <t>Never - automatic</t>
         </is>
       </c>
-      <c r="D18" s="49" t="inlineStr">
+      <c r="D18" s="51" t="inlineStr">
         <is>
           <t>Which orders took which boxes. The dashboard writes it.</t>
         </is>
       </c>
-      <c r="E18" s="54" t="n"/>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="52">
+      <c r="E18" s="56" t="n"/>
+    </row>
+    <row r="19" ht="15" customHeight="1" s="54">
       <c r="B19" s="10" t="inlineStr">
         <is>
           <t>MASTER</t>
         </is>
       </c>
-      <c r="C19" s="51" t="inlineStr">
+      <c r="C19" s="53" t="inlineStr">
         <is>
           <t>Rarely</t>
         </is>
       </c>
-      <c r="D19" s="51" t="inlineStr">
+      <c r="D19" s="53" t="inlineStr">
         <is>
           <t>Items, courier, reasons, movements, settings</t>
         </is>
       </c>
-      <c r="E19" s="54" t="n"/>
-    </row>
-    <row r="22" ht="15" customHeight="1" s="52">
+      <c r="E19" s="56" t="n"/>
+    </row>
+    <row r="22" ht="15" customHeight="1" s="54">
       <c r="B22" s="14" t="inlineStr">
         <is>
           <t>Your daily routine</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="52">
+    <row r="23" ht="15" customHeight="1" s="54">
       <c r="B23" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   1.  New shipment landed? Add its lines on SHIPMENTS first - one row per item.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="52">
+    <row r="24" ht="15" customHeight="1" s="54">
       <c r="B24" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   2.  Open MOVES. Type the Date and Shipment No, then pick the Movement.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="52">
+    <row r="25" ht="15" customHeight="1" s="54">
       <c r="B25" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   3.  Read the 'What to fill' column. It names every field that movement needs - fill only those.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="52">
+    <row r="26" ht="15" customHeight="1" s="54">
       <c r="B26" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   4.  Quantities go in the In column or the Out column, never both. The column tells you which.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="15" customHeight="1" s="52">
+    <row r="27" ht="15" customHeight="1" s="54">
       <c r="B27" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   5.  Check the last column shows OK on every new row. Save the file.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1" s="52">
+    <row r="28" ht="15" customHeight="1" s="54">
       <c r="B28" s="15" t="n"/>
     </row>
-    <row r="29" ht="15" customHeight="1" s="52">
+    <row r="29" ht="15" customHeight="1" s="54">
       <c r="B29" s="14" t="inlineStr">
         <is>
           <t>Made a mistake?</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="15" customHeight="1" s="52">
+    <row r="30" ht="15" customHeight="1" s="54">
       <c r="B30" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Set Void to Yes on that row. It is ignored everywhere and stays visible for audit. Never delete a row.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="15" customHeight="1" s="52">
+    <row r="31" ht="15" customHeight="1" s="54">
       <c r="B31" s="15" t="n"/>
     </row>
-    <row r="32" ht="15" customHeight="1" s="52">
+    <row r="32" ht="15" customHeight="1" s="54">
       <c r="B32" s="14" t="inlineStr">
         <is>
           <t>Rules that never change</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="15" customHeight="1" s="52">
+    <row r="33" ht="15" customHeight="1" s="54">
       <c r="B33" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Items are tracked inside the store. Once boxes go to the courier, quantities are tracked by shipment.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1" s="52">
+    <row r="34" ht="15" customHeight="1" s="54">
       <c r="B34" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Returns: enter Returned (no item), then split it the same day into Return to Saleable and Return to Scrap.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1" s="52">
+    <row r="35" ht="15" customHeight="1" s="54">
       <c r="B35" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Orders are counts, never order numbers. Order numbers appear only on DISPATCH, written automatically.</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="15" customHeight="1" s="52">
+    <row r="36" ht="15" customHeight="1" s="54">
       <c r="B36" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   A physical count never changes stock. Post a Count Adjustment in MOVES with a reason instead.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="15" customHeight="1" s="52">
+    <row r="37" ht="15" customHeight="1" s="54">
       <c r="B37" s="15" t="n"/>
     </row>
-    <row r="38" ht="15" customHeight="1" s="52">
+    <row r="38" ht="15" customHeight="1" s="54">
       <c r="B38" s="14" t="inlineStr">
         <is>
           <t>Growing this file</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="15" customHeight="1" s="52">
+    <row r="39" ht="15" customHeight="1" s="54">
       <c r="B39" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   New item, courier or reason  -&gt;  add a row on MASTER.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="15" customHeight="1" s="52">
+    <row r="40" ht="15" customHeight="1" s="54">
       <c r="B40" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   New kind of movement  -&gt;  add a row to the Movement Types table on MASTER. Nothing else changes.</t>
@@ -1602,59 +1602,59 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB31"/>
+  <dimension ref="A1:AB32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col width="2" customWidth="1" style="52" min="1" max="1"/>
-    <col width="49.5703125" customWidth="1" style="52" min="2" max="2"/>
-    <col width="24" customWidth="1" style="52" min="3" max="3"/>
-    <col width="9" customWidth="1" style="52" min="4" max="4"/>
-    <col width="2" customWidth="1" style="52" min="5" max="5"/>
-    <col width="10" customWidth="1" style="52" min="6" max="6"/>
-    <col width="8" customWidth="1" style="52" min="7" max="7"/>
-    <col width="2" customWidth="1" style="52" min="8" max="8"/>
-    <col width="12" customWidth="1" style="52" min="9" max="9"/>
-    <col width="9" customWidth="1" style="52" min="10" max="10"/>
-    <col width="8" customWidth="1" style="52" min="11" max="11"/>
-    <col width="2" customWidth="1" style="52" min="12" max="12"/>
-    <col width="22" customWidth="1" style="52" min="13" max="13"/>
-    <col width="10" customWidth="1" style="52" min="14" max="14"/>
-    <col width="2" customWidth="1" style="52" min="15" max="15"/>
-    <col width="25" customWidth="1" style="52" min="16" max="16"/>
-    <col width="30" customWidth="1" style="52" min="17" max="17"/>
-    <col width="7" customWidth="1" style="52" min="18" max="19"/>
-    <col width="9" customWidth="1" style="52" min="20" max="20"/>
-    <col width="8" customWidth="1" style="52" min="21" max="22"/>
-    <col width="7" customWidth="1" style="52" min="23" max="23"/>
-    <col width="2" customWidth="1" style="52" min="24" max="24"/>
-    <col width="16" customWidth="1" style="52" min="25" max="25"/>
-    <col width="10" customWidth="1" style="52" min="26" max="26"/>
-    <col width="9" customWidth="1" style="52" min="27" max="27"/>
-    <col width="8" customWidth="1" style="52" min="28" max="28"/>
+    <col width="2" customWidth="1" style="54" min="1" max="1"/>
+    <col width="49.5703125" customWidth="1" style="54" min="2" max="2"/>
+    <col width="24" customWidth="1" style="54" min="3" max="3"/>
+    <col width="9" customWidth="1" style="54" min="4" max="4"/>
+    <col width="2" customWidth="1" style="54" min="5" max="5"/>
+    <col width="10" customWidth="1" style="54" min="6" max="6"/>
+    <col width="8" customWidth="1" style="54" min="7" max="7"/>
+    <col width="2" customWidth="1" style="54" min="8" max="8"/>
+    <col width="12" customWidth="1" style="54" min="9" max="9"/>
+    <col width="9" customWidth="1" style="54" min="10" max="10"/>
+    <col width="8" customWidth="1" style="54" min="11" max="11"/>
+    <col width="2" customWidth="1" style="54" min="12" max="12"/>
+    <col width="22" customWidth="1" style="54" min="13" max="13"/>
+    <col width="10" customWidth="1" style="54" min="14" max="14"/>
+    <col width="2" customWidth="1" style="54" min="15" max="15"/>
+    <col width="25" customWidth="1" style="54" min="16" max="16"/>
+    <col width="30" customWidth="1" style="54" min="17" max="17"/>
+    <col width="7" customWidth="1" style="54" min="18" max="19"/>
+    <col width="9" customWidth="1" style="54" min="20" max="20"/>
+    <col width="8" customWidth="1" style="54" min="21" max="22"/>
+    <col width="7" customWidth="1" style="54" min="23" max="23"/>
+    <col width="2" customWidth="1" style="54" min="24" max="24"/>
+    <col width="16" customWidth="1" style="54" min="25" max="25"/>
+    <col width="10" customWidth="1" style="54" min="26" max="26"/>
+    <col width="9" customWidth="1" style="54" min="27" max="27"/>
+    <col width="8" customWidth="1" style="54" min="28" max="28"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="52">
+    <row r="1" ht="25.5" customHeight="1" s="54">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>MASTER  -  standards</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="52">
+    <row r="2" ht="15" customHeight="1" s="54">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Set once. Everything else reads from here.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="15.75" customHeight="1" s="52">
+    <row r="4" ht="15.75" customHeight="1" s="54">
       <c r="B4" s="16" t="inlineStr">
         <is>
           <t>SETTINGS</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="52">
+    <row r="5" ht="15" customHeight="1" s="54">
       <c r="B5" s="17" t="inlineStr">
         <is>
           <t>As-Of Date</t>
@@ -1664,7 +1664,7 @@
         <v>46258</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="52">
+    <row r="6" ht="15" customHeight="1" s="54">
       <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Courier holding limit (days)</t>
@@ -1674,7 +1674,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="52">
+    <row r="7" ht="15" customHeight="1" s="54">
       <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Shipment clearance target (days)</t>
@@ -1684,7 +1684,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="52">
+    <row r="8" ht="15" customHeight="1" s="54">
       <c r="B8" s="17" t="inlineStr">
         <is>
           <t>Loss % target</t>
@@ -1694,7 +1694,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="52">
+    <row r="9" ht="15" customHeight="1" s="54">
       <c r="B9" s="17" t="inlineStr">
         <is>
           <t>Count variance tolerance</t>
@@ -1704,7 +1704,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="52">
+    <row r="10" ht="15" customHeight="1" s="54">
       <c r="B10" s="17" t="inlineStr">
         <is>
           <t>Version</t>
@@ -1716,21 +1716,21 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="52">
+    <row r="12" ht="15" customHeight="1" s="54">
       <c r="B12" s="22" t="inlineStr">
         <is>
           <t>Yellow = the only cells you change here.  Holding limit 99 = no limit.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="15.75" customHeight="1" s="52">
+    <row r="14" ht="15.75" customHeight="1" s="54">
       <c r="B14" s="16" t="inlineStr">
         <is>
           <t>MASTER TABLES</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1" s="52">
+    <row r="15" ht="30" customHeight="1" s="54">
       <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Item Name</t>
@@ -1842,7 +1842,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" s="52">
+    <row r="16" ht="15" customHeight="1" s="54">
       <c r="B16" s="24" t="inlineStr">
         <is>
           <t>Mango Fas</t>
@@ -1954,7 +1954,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1" s="52">
+    <row r="17" ht="15" customHeight="1" s="54">
       <c r="B17" s="24" t="inlineStr">
         <is>
           <t>Mango Owais</t>
@@ -2066,7 +2066,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1" s="52">
+    <row r="18" ht="15" customHeight="1" s="54">
       <c r="B18" s="24" t="inlineStr">
         <is>
           <t>Fig Barshomi</t>
@@ -2178,7 +2178,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="52">
+    <row r="19" ht="15" customHeight="1" s="54">
       <c r="B19" s="24" t="inlineStr">
         <is>
           <t>Guava Banati</t>
@@ -2290,7 +2290,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="52">
+    <row r="20" ht="15" customHeight="1" s="54">
       <c r="B20" s="24" t="inlineStr">
         <is>
           <t>Mango White Sugar</t>
@@ -2377,7 +2377,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="52">
+    <row r="21" ht="15" customHeight="1" s="54">
       <c r="B21" s="24" t="inlineStr">
         <is>
           <t>Dates Barhi</t>
@@ -2444,7 +2444,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="52">
+    <row r="22" ht="15" customHeight="1" s="54">
       <c r="B22" s="24" t="inlineStr">
         <is>
           <t>Mango Trio Box</t>
@@ -2516,7 +2516,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="52">
+    <row r="23" ht="15" customHeight="1" s="54">
       <c r="B23" s="24" t="inlineStr">
         <is>
           <t>Mango Fons</t>
@@ -2583,7 +2583,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="52">
+    <row r="24" ht="15" customHeight="1" s="54">
       <c r="B24" s="24" t="inlineStr">
         <is>
           <t>Grapes Banati</t>
@@ -2650,7 +2650,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="52">
+    <row r="25" ht="15" customHeight="1" s="54">
       <c r="B25" s="24" t="inlineStr">
         <is>
           <t>Grapes Red</t>
@@ -2685,7 +2685,7 @@
       <c r="V25" s="24" t="n"/>
       <c r="W25" s="24" t="n"/>
     </row>
-    <row r="26" ht="15" customHeight="1" s="52">
+    <row r="26" ht="15" customHeight="1" s="54">
       <c r="B26" s="24" t="inlineStr">
         <is>
           <t>Mango Sediqa</t>
@@ -2720,7 +2720,7 @@
       <c r="V26" s="24" t="n"/>
       <c r="W26" s="24" t="n"/>
     </row>
-    <row r="27" ht="15" customHeight="1" s="52">
+    <row r="27" ht="15" customHeight="1" s="54">
       <c r="B27" s="24" t="inlineStr">
         <is>
           <t>Pear Banati</t>
@@ -2755,7 +2755,7 @@
       <c r="V27" s="24" t="n"/>
       <c r="W27" s="24" t="n"/>
     </row>
-    <row r="28" ht="15" customHeight="1" s="52">
+    <row r="28" ht="15" customHeight="1" s="54">
       <c r="B28" s="24" t="inlineStr">
         <is>
           <t>Cantaloupe</t>
@@ -2782,7 +2782,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1" s="52">
+    <row r="29" ht="15" customHeight="1" s="54">
       <c r="B29" s="24" t="inlineStr">
         <is>
           <t>Mango Naomi</t>
@@ -2814,7 +2814,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="15" customHeight="1" s="52">
+    <row r="30" ht="15" customHeight="1" s="54">
       <c r="B30" s="24" t="inlineStr">
         <is>
           <t>Mango Zebda</t>
@@ -2841,7 +2841,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="15" customHeight="1" s="52">
+    <row r="31" ht="15" customHeight="1" s="54">
       <c r="B31" s="24" t="inlineStr">
         <is>
           <t>Mango Timour</t>
@@ -2858,6 +2858,7 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
@@ -2879,42 +2880,42 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" style="52" min="1" max="1"/>
-    <col width="9" customWidth="1" style="52" min="2" max="2"/>
-    <col width="18.42578125" bestFit="1" customWidth="1" style="52" min="3" max="3"/>
-    <col width="9" customWidth="1" style="52" min="4" max="4"/>
-    <col width="20" customWidth="1" style="52" min="5" max="5"/>
-    <col width="12" customWidth="1" style="52" min="6" max="6"/>
-    <col width="20" customWidth="1" style="52" min="7" max="7"/>
-    <col width="23.140625" customWidth="1" style="52" min="8" max="8"/>
-    <col width="26" customWidth="1" style="52" min="9" max="9"/>
+    <col width="13" customWidth="1" style="54" min="1" max="1"/>
+    <col width="9" customWidth="1" style="54" min="2" max="2"/>
+    <col width="18.42578125" bestFit="1" customWidth="1" style="54" min="3" max="3"/>
+    <col width="9" customWidth="1" style="54" min="4" max="4"/>
+    <col width="20" customWidth="1" style="54" min="5" max="5"/>
+    <col width="12" customWidth="1" style="54" min="6" max="6"/>
+    <col width="20" customWidth="1" style="54" min="7" max="7"/>
+    <col width="23.140625" customWidth="1" style="54" min="8" max="8"/>
+    <col width="26" customWidth="1" style="54" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="52">
+    <row r="1" ht="25.5" customHeight="1" s="54">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>SHIPMENTS  -  what arrived</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="52">
+    <row r="2" ht="15" customHeight="1" s="54">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>One row per shipment and item. Filled once, when the shipment lands.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="52">
+    <row r="4" ht="15" customHeight="1" s="54">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>BLUE = you type it.   GREY = the workbook works it out.   RED = fix that row.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="31.5" customHeight="1" s="52">
+    <row r="6" ht="31.5" customHeight="1" s="54">
       <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Shipment No</t>
@@ -2961,7 +2962,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="52">
+    <row r="7" ht="15" customHeight="1" s="54">
       <c r="A7" t="inlineStr">
         <is>
           <t>Q-26-001</t>
@@ -2999,7 +3000,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="52">
+    <row r="8" ht="15" customHeight="1" s="54">
       <c r="A8" t="inlineStr">
         <is>
           <t>Q-26-001</t>
@@ -3037,7 +3038,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="52">
+    <row r="9" ht="15" customHeight="1" s="54">
       <c r="A9" t="inlineStr">
         <is>
           <t>Q-26-001</t>
@@ -3075,7 +3076,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="52">
+    <row r="10" ht="15" customHeight="1" s="54">
       <c r="A10" t="inlineStr">
         <is>
           <t>Q-26-001</t>
@@ -3113,7 +3114,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="52">
+    <row r="11" ht="15" customHeight="1" s="54">
       <c r="A11" t="inlineStr">
         <is>
           <t>Q-26-001</t>
@@ -3151,7 +3152,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="52">
+    <row r="12" ht="15" customHeight="1" s="54">
       <c r="A12" t="inlineStr">
         <is>
           <t>Q-26-001</t>
@@ -3189,7 +3190,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="52">
+    <row r="13" ht="15" customHeight="1" s="54">
       <c r="A13" t="inlineStr">
         <is>
           <t>Q-26-001</t>
@@ -3227,7 +3228,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="52">
+    <row r="14" ht="15" customHeight="1" s="54">
       <c r="A14" t="inlineStr">
         <is>
           <t>Q-26-001</t>
@@ -3265,7 +3266,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1" s="52">
+    <row r="15" ht="15" customHeight="1" s="54">
       <c r="A15" t="inlineStr">
         <is>
           <t>Q-26-001</t>
@@ -3303,7 +3304,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" s="52">
+    <row r="16" ht="15" customHeight="1" s="54">
       <c r="A16" t="inlineStr">
         <is>
           <t>Q-26-001</t>
@@ -3341,7 +3342,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1" s="52">
+    <row r="17" ht="15" customHeight="1" s="54">
       <c r="A17" t="inlineStr">
         <is>
           <t>Q-26-001</t>
@@ -3379,7 +3380,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1" s="52">
+    <row r="18" ht="15" customHeight="1" s="54">
       <c r="A18" t="inlineStr">
         <is>
           <t>Q-26-001</t>
@@ -3417,7 +3418,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="52">
+    <row r="19" ht="15" customHeight="1" s="54">
       <c r="A19" t="inlineStr">
         <is>
           <t>Q-26-001</t>
@@ -3455,7 +3456,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="52">
+    <row r="20" ht="15" customHeight="1" s="54">
       <c r="A20" t="inlineStr">
         <is>
           <t>Q-26-001</t>
@@ -3493,7 +3494,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="52">
+    <row r="21" ht="15" customHeight="1" s="54">
       <c r="A21" t="inlineStr">
         <is>
           <t>Q-26-001</t>
@@ -3531,7 +3532,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="52">
+    <row r="22" ht="15" customHeight="1" s="54">
       <c r="A22" t="inlineStr">
         <is>
           <t>Q-26-001</t>
@@ -3569,119 +3570,193 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="52"/>
-    <row r="24" ht="15" customHeight="1" s="52"/>
-    <row r="25" ht="15" customHeight="1" s="52"/>
-    <row r="26" ht="15" customHeight="1" s="52"/>
-    <row r="27" ht="15" customHeight="1" s="52"/>
-    <row r="28" ht="15" customHeight="1" s="52"/>
-    <row r="29" ht="15" customHeight="1" s="52"/>
-    <row r="30" ht="15" customHeight="1" s="52"/>
-    <row r="31" ht="15" customHeight="1" s="52"/>
-    <row r="32" ht="15" customHeight="1" s="52"/>
-    <row r="33" ht="15" customHeight="1" s="52"/>
-    <row r="34" ht="15" customHeight="1" s="52"/>
-    <row r="35" ht="15" customHeight="1" s="52"/>
-    <row r="36" ht="15" customHeight="1" s="52"/>
-    <row r="37" ht="15" customHeight="1" s="52"/>
-    <row r="38" ht="15" customHeight="1" s="52"/>
-    <row r="39" ht="15" customHeight="1" s="52"/>
-    <row r="40" ht="15" customHeight="1" s="52"/>
-    <row r="41" ht="15" customHeight="1" s="52"/>
-    <row r="42" ht="15" customHeight="1" s="52"/>
-    <row r="43" ht="15" customHeight="1" s="52"/>
-    <row r="44" ht="15" customHeight="1" s="52"/>
-    <row r="45" ht="15" customHeight="1" s="52"/>
-    <row r="46" ht="15" customHeight="1" s="52"/>
-    <row r="47" ht="15" customHeight="1" s="52"/>
-    <row r="48" ht="15" customHeight="1" s="52"/>
-    <row r="49" ht="15" customHeight="1" s="52"/>
-    <row r="50" ht="15" customHeight="1" s="52"/>
-    <row r="51" ht="15" customHeight="1" s="52"/>
-    <row r="52" ht="15" customHeight="1" s="52"/>
-    <row r="53" ht="15" customHeight="1" s="52"/>
-    <row r="54" ht="15" customHeight="1" s="52"/>
-    <row r="55" ht="15" customHeight="1" s="52"/>
-    <row r="56" ht="15" customHeight="1" s="52"/>
-    <row r="57" ht="15" customHeight="1" s="52"/>
-    <row r="58" ht="15" customHeight="1" s="52"/>
-    <row r="59" ht="15" customHeight="1" s="52"/>
-    <row r="60" ht="15" customHeight="1" s="52"/>
-    <row r="61" ht="15" customHeight="1" s="52"/>
-    <row r="62" ht="15" customHeight="1" s="52"/>
-    <row r="63" ht="15" customHeight="1" s="52"/>
-    <row r="64" ht="15" customHeight="1" s="52"/>
-    <row r="65" ht="15" customHeight="1" s="52"/>
-    <row r="66" ht="15" customHeight="1" s="52"/>
-    <row r="67" ht="15" customHeight="1" s="52"/>
-    <row r="68" ht="15" customHeight="1" s="52"/>
-    <row r="69" ht="15" customHeight="1" s="52"/>
-    <row r="70" ht="15" customHeight="1" s="52"/>
-    <row r="71" ht="15" customHeight="1" s="52"/>
-    <row r="72" ht="15" customHeight="1" s="52"/>
-    <row r="73" ht="15" customHeight="1" s="52"/>
-    <row r="74" ht="15" customHeight="1" s="52"/>
-    <row r="75" ht="15" customHeight="1" s="52"/>
-    <row r="76" ht="15" customHeight="1" s="52"/>
-    <row r="77" ht="15" customHeight="1" s="52"/>
-    <row r="78" ht="15" customHeight="1" s="52"/>
-    <row r="79" ht="15" customHeight="1" s="52"/>
-    <row r="80" ht="15" customHeight="1" s="52"/>
-    <row r="81" ht="15" customHeight="1" s="52"/>
-    <row r="82" ht="15" customHeight="1" s="52"/>
-    <row r="83" ht="15" customHeight="1" s="52"/>
-    <row r="84" ht="15" customHeight="1" s="52"/>
-    <row r="85" ht="15" customHeight="1" s="52"/>
-    <row r="86" ht="15" customHeight="1" s="52"/>
-    <row r="87" ht="15" customHeight="1" s="52"/>
-    <row r="88" ht="15" customHeight="1" s="52"/>
-    <row r="89" ht="15" customHeight="1" s="52"/>
-    <row r="90" ht="15" customHeight="1" s="52"/>
-    <row r="91" ht="15" customHeight="1" s="52"/>
-    <row r="92" ht="15" customHeight="1" s="52"/>
-    <row r="93" ht="15" customHeight="1" s="52"/>
-    <row r="94" ht="15" customHeight="1" s="52"/>
-    <row r="95" ht="15" customHeight="1" s="52"/>
-    <row r="96" ht="15" customHeight="1" s="52"/>
-    <row r="97" ht="15" customHeight="1" s="52"/>
-    <row r="98" ht="15" customHeight="1" s="52"/>
-    <row r="99" ht="15" customHeight="1" s="52"/>
-    <row r="100" ht="15" customHeight="1" s="52"/>
-    <row r="101" ht="15" customHeight="1" s="52"/>
-    <row r="102" ht="15" customHeight="1" s="52"/>
-    <row r="103" ht="15" customHeight="1" s="52"/>
-    <row r="104" ht="15" customHeight="1" s="52"/>
-    <row r="105" ht="15" customHeight="1" s="52"/>
-    <row r="106" ht="15" customHeight="1" s="52"/>
-    <row r="107" ht="15" customHeight="1" s="52"/>
-    <row r="108" ht="15" customHeight="1" s="52"/>
-    <row r="109" ht="15" customHeight="1" s="52"/>
-    <row r="110" ht="15" customHeight="1" s="52"/>
-    <row r="111" ht="15" customHeight="1" s="52"/>
-    <row r="112" ht="15" customHeight="1" s="52"/>
-    <row r="113" ht="15" customHeight="1" s="52"/>
-    <row r="114" ht="15" customHeight="1" s="52"/>
-    <row r="115" ht="15" customHeight="1" s="52"/>
-    <row r="116" ht="15" customHeight="1" s="52"/>
-    <row r="117" ht="15" customHeight="1" s="52"/>
-    <row r="118" ht="15" customHeight="1" s="52"/>
-    <row r="119" ht="15" customHeight="1" s="52"/>
-    <row r="120" ht="15" customHeight="1" s="52"/>
-    <row r="121" ht="15" customHeight="1" s="52"/>
-    <row r="122" ht="15" customHeight="1" s="52"/>
-    <row r="123" ht="15" customHeight="1" s="52"/>
-    <row r="124" ht="15" customHeight="1" s="52"/>
-    <row r="125" ht="15" customHeight="1" s="52"/>
-    <row r="126" ht="15" customHeight="1" s="52"/>
-    <row r="127" ht="15" customHeight="1" s="52"/>
-    <row r="128" ht="15" customHeight="1" s="52"/>
-    <row r="129" ht="15" customHeight="1" s="52"/>
-    <row r="130" ht="15" customHeight="1" s="52"/>
-    <row r="131" ht="15" customHeight="1" s="52"/>
-    <row r="132" ht="15" customHeight="1" s="52"/>
-    <row r="133" ht="15" customHeight="1" s="52"/>
-    <row r="134" ht="15" customHeight="1" s="52"/>
-    <row r="135" ht="15" customHeight="1" s="52"/>
+    <row r="23" ht="15" customHeight="1" s="54">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Q-26-002</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="C23" s="57" t="n">
+        <v>46261</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Grapes Banati</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>2</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>EG-FG-GRP-01-02-01-01</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1" s="54">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Q-26-002</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="C24" s="57" t="n">
+        <v>46261</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Fig Barshomi</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>EG-FG-FIG-01-02-01-01</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1" s="54"/>
+    <row r="26" ht="15" customHeight="1" s="54"/>
+    <row r="27" ht="15" customHeight="1" s="54"/>
+    <row r="28" ht="15" customHeight="1" s="54"/>
+    <row r="29" ht="15" customHeight="1" s="54"/>
+    <row r="30" ht="15" customHeight="1" s="54"/>
+    <row r="31" ht="15" customHeight="1" s="54"/>
+    <row r="32" ht="15" customHeight="1" s="54"/>
+    <row r="33" ht="15" customHeight="1" s="54"/>
+    <row r="34" ht="15" customHeight="1" s="54"/>
+    <row r="35" ht="15" customHeight="1" s="54"/>
+    <row r="36" ht="15" customHeight="1" s="54"/>
+    <row r="37" ht="15" customHeight="1" s="54"/>
+    <row r="38" ht="15" customHeight="1" s="54"/>
+    <row r="39" ht="15" customHeight="1" s="54"/>
+    <row r="40" ht="15" customHeight="1" s="54"/>
+    <row r="41" ht="15" customHeight="1" s="54"/>
+    <row r="42" ht="15" customHeight="1" s="54"/>
+    <row r="43" ht="15" customHeight="1" s="54"/>
+    <row r="44" ht="15" customHeight="1" s="54"/>
+    <row r="45" ht="15" customHeight="1" s="54"/>
+    <row r="46" ht="15" customHeight="1" s="54"/>
+    <row r="47" ht="15" customHeight="1" s="54"/>
+    <row r="48" ht="15" customHeight="1" s="54"/>
+    <row r="49" ht="15" customHeight="1" s="54"/>
+    <row r="50" ht="15" customHeight="1" s="54"/>
+    <row r="51" ht="15" customHeight="1" s="54"/>
+    <row r="52" ht="15" customHeight="1" s="54"/>
+    <row r="53" ht="15" customHeight="1" s="54"/>
+    <row r="54" ht="15" customHeight="1" s="54"/>
+    <row r="55" ht="15" customHeight="1" s="54"/>
+    <row r="56" ht="15" customHeight="1" s="54"/>
+    <row r="57" ht="15" customHeight="1" s="54"/>
+    <row r="58" ht="15" customHeight="1" s="54"/>
+    <row r="59" ht="15" customHeight="1" s="54"/>
+    <row r="60" ht="15" customHeight="1" s="54"/>
+    <row r="61" ht="15" customHeight="1" s="54"/>
+    <row r="62" ht="15" customHeight="1" s="54"/>
+    <row r="63" ht="15" customHeight="1" s="54"/>
+    <row r="64" ht="15" customHeight="1" s="54"/>
+    <row r="65" ht="15" customHeight="1" s="54"/>
+    <row r="66" ht="15" customHeight="1" s="54"/>
+    <row r="67" ht="15" customHeight="1" s="54"/>
+    <row r="68" ht="15" customHeight="1" s="54"/>
+    <row r="69" ht="15" customHeight="1" s="54"/>
+    <row r="70" ht="15" customHeight="1" s="54"/>
+    <row r="71" ht="15" customHeight="1" s="54"/>
+    <row r="72" ht="15" customHeight="1" s="54"/>
+    <row r="73" ht="15" customHeight="1" s="54"/>
+    <row r="74" ht="15" customHeight="1" s="54"/>
+    <row r="75" ht="15" customHeight="1" s="54"/>
+    <row r="76" ht="15" customHeight="1" s="54"/>
+    <row r="77" ht="15" customHeight="1" s="54"/>
+    <row r="78" ht="15" customHeight="1" s="54"/>
+    <row r="79" ht="15" customHeight="1" s="54"/>
+    <row r="80" ht="15" customHeight="1" s="54"/>
+    <row r="81" ht="15" customHeight="1" s="54"/>
+    <row r="82" ht="15" customHeight="1" s="54"/>
+    <row r="83" ht="15" customHeight="1" s="54"/>
+    <row r="84" ht="15" customHeight="1" s="54"/>
+    <row r="85" ht="15" customHeight="1" s="54"/>
+    <row r="86" ht="15" customHeight="1" s="54"/>
+    <row r="87" ht="15" customHeight="1" s="54"/>
+    <row r="88" ht="15" customHeight="1" s="54"/>
+    <row r="89" ht="15" customHeight="1" s="54"/>
+    <row r="90" ht="15" customHeight="1" s="54"/>
+    <row r="91" ht="15" customHeight="1" s="54"/>
+    <row r="92" ht="15" customHeight="1" s="54"/>
+    <row r="93" ht="15" customHeight="1" s="54"/>
+    <row r="94" ht="15" customHeight="1" s="54"/>
+    <row r="95" ht="15" customHeight="1" s="54"/>
+    <row r="96" ht="15" customHeight="1" s="54"/>
+    <row r="97" ht="15" customHeight="1" s="54"/>
+    <row r="98" ht="15" customHeight="1" s="54"/>
+    <row r="99" ht="15" customHeight="1" s="54"/>
+    <row r="100" ht="15" customHeight="1" s="54"/>
+    <row r="101" ht="15" customHeight="1" s="54"/>
+    <row r="102" ht="15" customHeight="1" s="54"/>
+    <row r="103" ht="15" customHeight="1" s="54"/>
+    <row r="104" ht="15" customHeight="1" s="54"/>
+    <row r="105" ht="15" customHeight="1" s="54"/>
+    <row r="106" ht="15" customHeight="1" s="54"/>
+    <row r="107" ht="15" customHeight="1" s="54"/>
+    <row r="108" ht="15" customHeight="1" s="54"/>
+    <row r="109" ht="15" customHeight="1" s="54"/>
+    <row r="110" ht="15" customHeight="1" s="54"/>
+    <row r="111" ht="15" customHeight="1" s="54"/>
+    <row r="112" ht="15" customHeight="1" s="54"/>
+    <row r="113" ht="15" customHeight="1" s="54"/>
+    <row r="114" ht="15" customHeight="1" s="54"/>
+    <row r="115" ht="15" customHeight="1" s="54"/>
+    <row r="116" ht="15" customHeight="1" s="54"/>
+    <row r="117" ht="15" customHeight="1" s="54"/>
+    <row r="118" ht="15" customHeight="1" s="54"/>
+    <row r="119" ht="15" customHeight="1" s="54"/>
+    <row r="120" ht="15" customHeight="1" s="54"/>
+    <row r="121" ht="15" customHeight="1" s="54"/>
+    <row r="122" ht="15" customHeight="1" s="54"/>
+    <row r="123" ht="15" customHeight="1" s="54"/>
+    <row r="124" ht="15" customHeight="1" s="54"/>
+    <row r="125" ht="15" customHeight="1" s="54"/>
+    <row r="126" ht="15" customHeight="1" s="54"/>
+    <row r="127" ht="15" customHeight="1" s="54"/>
+    <row r="128" ht="15" customHeight="1" s="54"/>
+    <row r="129" ht="15" customHeight="1" s="54"/>
+    <row r="130" ht="15" customHeight="1" s="54"/>
+    <row r="131" ht="15" customHeight="1" s="54"/>
+    <row r="132" ht="15" customHeight="1" s="54"/>
+    <row r="133" ht="15" customHeight="1" s="54"/>
+    <row r="134" ht="15" customHeight="1" s="54"/>
+    <row r="135" ht="15" customHeight="1" s="54"/>
   </sheetData>
   <conditionalFormatting sqref="I7:I9000">
     <cfRule type="expression" priority="2" dxfId="0">
@@ -3720,47 +3795,47 @@
   <dimension ref="A1:S31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" style="52" min="1" max="1"/>
-    <col width="12" customWidth="1" style="52" min="2" max="2"/>
-    <col width="24.85546875" customWidth="1" style="52" min="3" max="3"/>
-    <col width="34" customWidth="1" style="52" min="4" max="4"/>
-    <col width="20" customWidth="1" style="52" min="5" max="5"/>
-    <col width="8" customWidth="1" style="52" min="6" max="7"/>
-    <col width="8.42578125" customWidth="1" style="52" min="8" max="8"/>
-    <col width="13" customWidth="1" style="52" min="9" max="9"/>
-    <col width="19" customWidth="1" style="52" min="10" max="10"/>
-    <col width="18" customWidth="1" style="52" min="11" max="11"/>
-    <col width="7" customWidth="1" style="52" min="12" max="12"/>
-    <col width="23" customWidth="1" style="52" min="13" max="13"/>
-    <col width="9" customWidth="1" style="52" min="14" max="14"/>
-    <col width="7" customWidth="1" style="52" min="15" max="15"/>
-    <col width="17" customWidth="1" style="52" min="16" max="16"/>
-    <col width="13" customWidth="1" style="52" min="17" max="17"/>
-    <col width="17" customWidth="1" style="52" min="18" max="18"/>
+    <col width="11" customWidth="1" style="54" min="1" max="1"/>
+    <col width="12" customWidth="1" style="54" min="2" max="2"/>
+    <col width="24.85546875" customWidth="1" style="54" min="3" max="3"/>
+    <col width="34" customWidth="1" style="54" min="4" max="4"/>
+    <col width="20" customWidth="1" style="54" min="5" max="5"/>
+    <col width="8" customWidth="1" style="54" min="6" max="7"/>
+    <col width="8.42578125" customWidth="1" style="54" min="8" max="8"/>
+    <col width="13" customWidth="1" style="54" min="9" max="9"/>
+    <col width="19" customWidth="1" style="54" min="10" max="10"/>
+    <col width="18" customWidth="1" style="54" min="11" max="11"/>
+    <col width="7" customWidth="1" style="54" min="12" max="12"/>
+    <col width="23" customWidth="1" style="54" min="13" max="13"/>
+    <col width="9" customWidth="1" style="54" min="14" max="14"/>
+    <col width="7" customWidth="1" style="54" min="15" max="15"/>
+    <col width="17" customWidth="1" style="54" min="16" max="16"/>
+    <col width="13" customWidth="1" style="54" min="17" max="17"/>
+    <col width="17" customWidth="1" style="54" min="18" max="18"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="52">
+    <row r="1" ht="25.5" customHeight="1" s="54">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>MOVES  -  the daily log</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="52">
+    <row r="2" ht="15" customHeight="1" s="54">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Pick the Movement first. The next column tells you exactly which fields to fill. Leave everything else blank.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="52">
+    <row r="4" ht="15" customHeight="1" s="54">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Made a mistake? Set Void to Yes. The row is ignored everywhere and stays visible. Never delete a row.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="31.5" customHeight="1" s="52">
+    <row r="6" ht="31.5" customHeight="1" s="54">
       <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Date</t>
@@ -3857,7 +3932,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="52">
+    <row r="7" ht="15" customHeight="1" s="54">
       <c r="A7" s="34" t="n">
         <v>46258</v>
       </c>
@@ -3916,7 +3991,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="52">
+    <row r="8" ht="15" customHeight="1" s="54">
       <c r="A8" s="34" t="n">
         <v>46258</v>
       </c>
@@ -3975,7 +4050,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="52">
+    <row r="9" ht="15" customHeight="1" s="54">
       <c r="A9" s="34" t="n">
         <v>46258</v>
       </c>
@@ -4034,7 +4109,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="52">
+    <row r="10" ht="15" customHeight="1" s="54">
       <c r="A10" s="34" t="n">
         <v>46258</v>
       </c>
@@ -4093,7 +4168,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="52">
+    <row r="11" ht="15" customHeight="1" s="54">
       <c r="A11" s="34" t="n">
         <v>46258</v>
       </c>
@@ -4152,7 +4227,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="52">
+    <row r="12" ht="15" customHeight="1" s="54">
       <c r="A12" s="34" t="n">
         <v>46258</v>
       </c>
@@ -4211,7 +4286,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="52">
+    <row r="13" ht="15" customHeight="1" s="54">
       <c r="A13" s="34" t="n">
         <v>46258</v>
       </c>
@@ -4270,7 +4345,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="52">
+    <row r="14" ht="15" customHeight="1" s="54">
       <c r="A14" s="34" t="n">
         <v>46258</v>
       </c>
@@ -4329,7 +4404,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1" s="52">
+    <row r="15" ht="15" customHeight="1" s="54">
       <c r="A15" s="34" t="n">
         <v>46258</v>
       </c>
@@ -4388,7 +4463,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" s="52">
+    <row r="16" ht="15" customHeight="1" s="54">
       <c r="A16" s="34" t="n">
         <v>46258</v>
       </c>
@@ -4447,7 +4522,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1" s="52">
+    <row r="17" ht="15" customHeight="1" s="54">
       <c r="A17" s="34" t="n">
         <v>46258</v>
       </c>
@@ -4506,7 +4581,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1" s="52">
+    <row r="18" ht="15" customHeight="1" s="54">
       <c r="A18" s="34" t="n">
         <v>46258</v>
       </c>
@@ -4565,7 +4640,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="52">
+    <row r="19" ht="15" customHeight="1" s="54">
       <c r="A19" s="34" t="n">
         <v>46258</v>
       </c>
@@ -4624,7 +4699,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="52">
+    <row r="20" ht="15" customHeight="1" s="54">
       <c r="A20" s="34" t="n">
         <v>46258</v>
       </c>
@@ -4683,7 +4758,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="52">
+    <row r="21" ht="15" customHeight="1" s="54">
       <c r="A21" s="34" t="n">
         <v>46258</v>
       </c>
@@ -4742,7 +4817,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="52">
+    <row r="22" ht="15" customHeight="1" s="54">
       <c r="A22" s="34" t="n">
         <v>46258</v>
       </c>
@@ -4801,7 +4876,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="52">
+    <row r="23" ht="15" customHeight="1" s="54">
       <c r="A23" s="34" t="n">
         <v>46258</v>
       </c>
@@ -4864,7 +4939,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="52">
+    <row r="24" ht="15" customHeight="1" s="54">
       <c r="A24" s="34" t="n">
         <v>46258</v>
       </c>
@@ -4927,7 +5002,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="52">
+    <row r="25" ht="15" customHeight="1" s="54">
       <c r="A25" s="34" t="n">
         <v>46258</v>
       </c>
@@ -4990,7 +5065,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="52">
+    <row r="26" ht="15" customHeight="1" s="54">
       <c r="A26" s="34" t="n">
         <v>46258</v>
       </c>
@@ -5053,7 +5128,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="15" customHeight="1" s="52">
+    <row r="27" ht="15" customHeight="1" s="54">
       <c r="A27" s="34" t="n">
         <v>46258</v>
       </c>
@@ -5120,7 +5195,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1" s="52">
+    <row r="28" ht="15" customHeight="1" s="54">
       <c r="A28" s="34" t="n">
         <v>46258</v>
       </c>
@@ -5184,7 +5259,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="57" t="n">
+      <c r="A29" s="49" t="n">
         <v>46260</v>
       </c>
       <c r="B29" t="inlineStr">
@@ -5248,7 +5323,7 @@
           <t>admin</t>
         </is>
       </c>
-      <c r="R29" s="58" t="n">
+      <c r="R29" s="50" t="n">
         <v>46260.9423210301</v>
       </c>
       <c r="S29" t="inlineStr">
@@ -5258,7 +5333,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="57" t="n">
+      <c r="A30" s="49" t="n">
         <v>46260</v>
       </c>
       <c r="B30" t="inlineStr">
@@ -5322,7 +5397,7 @@
           <t>admin</t>
         </is>
       </c>
-      <c r="R30" s="58" t="n">
+      <c r="R30" s="50" t="n">
         <v>46260.95209969908</v>
       </c>
       <c r="S30" t="inlineStr">
@@ -5332,7 +5407,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="57" t="n">
+      <c r="A31" s="49" t="n">
         <v>46260</v>
       </c>
       <c r="B31" t="inlineStr">
@@ -5396,7 +5471,7 @@
           <t>admin</t>
         </is>
       </c>
-      <c r="R31" s="58" t="n">
+      <c r="R31" s="50" t="n">
         <v>46260.96085467593</v>
       </c>
       <c r="S31" t="inlineStr">
@@ -5478,38 +5553,38 @@
   <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" style="52" min="1" max="1"/>
-    <col width="12" customWidth="1" style="52" min="2" max="2"/>
-    <col width="20" customWidth="1" style="52" min="3" max="3"/>
-    <col width="12" customWidth="1" style="52" min="4" max="4"/>
-    <col width="13" customWidth="1" style="52" min="5" max="5"/>
-    <col width="18" customWidth="1" style="52" min="6" max="6"/>
-    <col width="23" customWidth="1" style="52" min="7" max="7"/>
-    <col width="26" customWidth="1" style="52" min="8" max="8"/>
+    <col width="11" customWidth="1" style="54" min="1" max="1"/>
+    <col width="12" customWidth="1" style="54" min="2" max="2"/>
+    <col width="20" customWidth="1" style="54" min="3" max="3"/>
+    <col width="12" customWidth="1" style="54" min="4" max="4"/>
+    <col width="13" customWidth="1" style="54" min="5" max="5"/>
+    <col width="18" customWidth="1" style="54" min="6" max="6"/>
+    <col width="23" customWidth="1" style="54" min="7" max="7"/>
+    <col width="26" customWidth="1" style="54" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="52">
+    <row r="1" ht="25.5" customHeight="1" s="54">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>COUNT  -  physical stock check</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="52">
+    <row r="2" ht="15" customHeight="1" s="54">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Weekly or spot check. A count never changes stock - post a Count Adjustment in MOVES to correct it.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="52">
+    <row r="4" ht="15" customHeight="1" s="54">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Counted By is optional. Variance is calculated on the dashboard, not here.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="31.5" customHeight="1" s="52">
+    <row r="6" ht="31.5" customHeight="1" s="54">
       <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Date</t>
@@ -5551,16 +5626,16 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="52"/>
-    <row r="8" ht="15" customHeight="1" s="52"/>
-    <row r="9" ht="15" customHeight="1" s="52"/>
-    <row r="10" ht="15" customHeight="1" s="52"/>
-    <row r="11" ht="15" customHeight="1" s="52"/>
-    <row r="12" ht="15" customHeight="1" s="52"/>
-    <row r="13" ht="15" customHeight="1" s="52"/>
-    <row r="14" ht="15" customHeight="1" s="52"/>
-    <row r="15" ht="15" customHeight="1" s="52"/>
-    <row r="16" ht="15" customHeight="1" s="52"/>
+    <row r="7" ht="15" customHeight="1" s="54"/>
+    <row r="8" ht="15" customHeight="1" s="54"/>
+    <row r="9" ht="15" customHeight="1" s="54"/>
+    <row r="10" ht="15" customHeight="1" s="54"/>
+    <row r="11" ht="15" customHeight="1" s="54"/>
+    <row r="12" ht="15" customHeight="1" s="54"/>
+    <row r="13" ht="15" customHeight="1" s="54"/>
+    <row r="14" ht="15" customHeight="1" s="54"/>
+    <row r="15" ht="15" customHeight="1" s="54"/>
+    <row r="16" ht="15" customHeight="1" s="54"/>
   </sheetData>
   <conditionalFormatting sqref="H7:H9000">
     <cfRule type="expression" priority="2" dxfId="0">
@@ -5595,38 +5670,38 @@
   <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" style="52" min="1" max="1"/>
-    <col width="9" customWidth="1" style="52" min="2" max="2"/>
-    <col width="12" customWidth="1" style="52" min="3" max="4"/>
-    <col width="20" customWidth="1" style="52" min="5" max="5"/>
-    <col width="8" customWidth="1" style="52" min="6" max="6"/>
-    <col width="13" customWidth="1" style="52" min="7" max="7"/>
-    <col width="23" customWidth="1" style="52" min="8" max="8"/>
-    <col width="26" customWidth="1" style="52" min="9" max="9"/>
+    <col width="11" customWidth="1" style="54" min="1" max="1"/>
+    <col width="9" customWidth="1" style="54" min="2" max="2"/>
+    <col width="12" customWidth="1" style="54" min="3" max="4"/>
+    <col width="20" customWidth="1" style="54" min="5" max="5"/>
+    <col width="8" customWidth="1" style="54" min="6" max="6"/>
+    <col width="13" customWidth="1" style="54" min="7" max="7"/>
+    <col width="23" customWidth="1" style="54" min="8" max="8"/>
+    <col width="26" customWidth="1" style="54" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="52">
+    <row r="1" ht="25.5" customHeight="1" s="54">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>DISPATCH  -  written by the dashboard</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="52">
+    <row r="2" ht="15" customHeight="1" s="54">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>One row per order line dispatched. You do not type here - the Dispatch tab writes it when you confirm.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="52">
+    <row r="4" ht="15" customHeight="1" s="54">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>EXAMPLE row - delete it before you start.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="31.5" customHeight="1" s="52">
+    <row r="6" ht="31.5" customHeight="1" s="54">
       <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Date</t>
@@ -5673,7 +5748,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="52">
+    <row r="7" ht="15" customHeight="1" s="54">
       <c r="A7" s="44" t="n"/>
       <c r="B7" s="45" t="n"/>
       <c r="C7" s="45" t="n"/>
@@ -5852,13 +5927,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DE7AC01-F156-4D0F-9089-DB8057DC708F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{84D81202-C690-4C4F-88F9-3292E0CAE465}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{65402AA4-0D3A-49D1-83D3-656FEE7755F3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47637D39-ED47-498C-A4AB-103DA6A3A42F}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{176B3713-A76A-493A-8A45-CDF2C12E28DC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD51E8E6-1104-4166-8DBA-849C5D54171E}"/>
 </file>
</xml_diff>

<commit_message>
as-of never falls behind today
</commit_message>
<xml_diff>
--- a/Stock_Control/INRIPE_Stock_Entry_v1.xlsx
+++ b/Stock_Control/INRIPE_Stock_Entry_v1.xlsx
@@ -41,8 +41,8 @@
     <numFmt numFmtId="165" formatCode="dd\-mmm\-yy\ hh:mm"/>
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
     <numFmt numFmtId="167" formatCode="dd\-mmm\-yy"/>
-    <numFmt numFmtId="168" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="169" formatCode="dd-mmm-yy"/>
+    <numFmt numFmtId="168" formatCode="dd-mmm-yy"/>
+    <numFmt numFmtId="169" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="23">
     <font>
@@ -362,7 +362,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -492,6 +492,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1022,8 +1023,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="tblShipment" displayName="tblShipment" ref="A6:I24" headerRowCount="1">
-  <autoFilter ref="A6:I24"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="tblShipment" displayName="tblShipment" ref="A6:I22" headerRowCount="1">
+  <autoFilter ref="A6:I22"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Shipment No"/>
     <tableColumn id="2" name="Market"/>
@@ -1035,7 +1036,7 @@
     <tableColumn id="8" name="Item Code"/>
     <tableColumn id="9" name="Check"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
 </table>
 </file>
 
@@ -1602,7 +1603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB32"/>
+  <dimension ref="A1:AB31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="54" min="1" max="1"/>
@@ -2858,7 +2859,6 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
@@ -2880,7 +2880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="54" min="1" max="1"/>
@@ -2973,7 +2973,7 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="C7" s="48" t="n">
+      <c r="C7" s="58" t="n">
         <v>46258</v>
       </c>
       <c r="D7" t="inlineStr">
@@ -3011,7 +3011,7 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="C8" s="48" t="n">
+      <c r="C8" s="58" t="n">
         <v>46258</v>
       </c>
       <c r="D8" t="inlineStr">
@@ -3049,7 +3049,7 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="C9" s="48" t="n">
+      <c r="C9" s="58" t="n">
         <v>46258</v>
       </c>
       <c r="D9" t="inlineStr">
@@ -3087,7 +3087,7 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="C10" s="48" t="n">
+      <c r="C10" s="58" t="n">
         <v>46258</v>
       </c>
       <c r="D10" t="inlineStr">
@@ -3125,7 +3125,7 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="C11" s="48" t="n">
+      <c r="C11" s="58" t="n">
         <v>46258</v>
       </c>
       <c r="D11" t="inlineStr">
@@ -3163,7 +3163,7 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="C12" s="48" t="n">
+      <c r="C12" s="58" t="n">
         <v>46258</v>
       </c>
       <c r="D12" t="inlineStr">
@@ -3201,7 +3201,7 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="C13" s="48" t="n">
+      <c r="C13" s="58" t="n">
         <v>46258</v>
       </c>
       <c r="D13" t="inlineStr">
@@ -3239,7 +3239,7 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="C14" s="48" t="n">
+      <c r="C14" s="58" t="n">
         <v>46258</v>
       </c>
       <c r="D14" t="inlineStr">
@@ -3277,7 +3277,7 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="C15" s="48" t="n">
+      <c r="C15" s="58" t="n">
         <v>46258</v>
       </c>
       <c r="D15" t="inlineStr">
@@ -3315,7 +3315,7 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="C16" s="48" t="n">
+      <c r="C16" s="58" t="n">
         <v>46258</v>
       </c>
       <c r="D16" t="inlineStr">
@@ -3353,7 +3353,7 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="C17" s="48" t="n">
+      <c r="C17" s="58" t="n">
         <v>46258</v>
       </c>
       <c r="D17" t="inlineStr">
@@ -3391,7 +3391,7 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="C18" s="48" t="n">
+      <c r="C18" s="58" t="n">
         <v>46258</v>
       </c>
       <c r="D18" t="inlineStr">
@@ -3429,7 +3429,7 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="C19" s="48" t="n">
+      <c r="C19" s="58" t="n">
         <v>46258</v>
       </c>
       <c r="D19" t="inlineStr">
@@ -3467,7 +3467,7 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="C20" s="48" t="n">
+      <c r="C20" s="58" t="n">
         <v>46258</v>
       </c>
       <c r="D20" t="inlineStr">
@@ -3505,7 +3505,7 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="C21" s="48" t="n">
+      <c r="C21" s="58" t="n">
         <v>46258</v>
       </c>
       <c r="D21" t="inlineStr">
@@ -3543,7 +3543,7 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="C22" s="48" t="n">
+      <c r="C22" s="58" t="n">
         <v>46258</v>
       </c>
       <c r="D22" t="inlineStr">
@@ -3570,82 +3570,8 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="54">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Q-26-002</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Qatar</t>
-        </is>
-      </c>
-      <c r="C23" s="57" t="n">
-        <v>46261</v>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Grapes Banati</t>
-        </is>
-      </c>
-      <c r="F23" t="n">
-        <v>2</v>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>EG-FG-GRP-01-02-01-01</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15" customHeight="1" s="54">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Q-26-002</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Qatar</t>
-        </is>
-      </c>
-      <c r="C24" s="57" t="n">
-        <v>46261</v>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Fig Barshomi</t>
-        </is>
-      </c>
-      <c r="F24" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>EG-FG-FIG-01-02-01-01</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
+    <row r="23" ht="15" customHeight="1" s="54"/>
+    <row r="24" ht="15" customHeight="1" s="54"/>
     <row r="25" ht="15" customHeight="1" s="54"/>
     <row r="26" ht="15" customHeight="1" s="54"/>
     <row r="27" ht="15" customHeight="1" s="54"/>
@@ -5927,13 +5853,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{84D81202-C690-4C4F-88F9-3292E0CAE465}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E62F00BC-2969-4C87-BF1B-143542CAAA8B}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47637D39-ED47-498C-A4AB-103DA6A3A42F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{433234C5-CD61-4E2C-BE36-BF3250E08EAC}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD51E8E6-1104-4166-8DBA-849C5D54171E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0EBBA444-FA7E-4F1E-8420-D2094FE9A024}"/>
 </file>
</xml_diff>

<commit_message>
voided lines stay visible
</commit_message>
<xml_diff>
--- a/Stock_Control/INRIPE_Stock_Entry_v1.xlsx
+++ b/Stock_Control/INRIPE_Stock_Entry_v1.xlsx
@@ -1055,8 +1055,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="tblMoves" displayName="tblMoves" ref="A6:S46" headerRowCount="1">
-  <autoFilter ref="A6:S46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="tblMoves" displayName="tblMoves" ref="A6:S48" headerRowCount="1">
+  <autoFilter ref="A6:S48"/>
   <tableColumns count="19">
     <tableColumn id="1" name="Date"/>
     <tableColumn id="2" name="Shipment No"/>
@@ -4226,7 +4226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S46"/>
+  <dimension ref="A1:S48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="55" min="1" max="1"/>
@@ -6889,6 +6889,149 @@
         <v>46263.73066756944</v>
       </c>
       <c r="S46" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="59" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Q-26-003</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Scrap</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>OUT   fill: Item  Out  Reason</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Mango Owais</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>2</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>EG-FG-MNG-12-02-01-01</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="O47" t="n">
+        <v>2</v>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>Q-20260829-0009</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="R47" s="61" t="n">
+        <v>46263.77142931713</v>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="59" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Q-26-003</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>IN   fill: Item  In  Courier  Reason</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Mango Owais</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>6</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>WareOne</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Customer Refused</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>voided by admin 29 Aug 18:36</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>EG-FG-MNG-12-02-01-01</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="O48" t="n">
+        <v>6</v>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>Q-20260829-0010</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="R48" s="61" t="n">
+        <v>46263.7751134838</v>
+      </c>
+      <c r="S48" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -7341,13 +7484,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E563BDE5-E042-4CA8-AC57-F2D89BB94699}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{659E6CF3-0F4A-409D-AD14-4AE7D4F368A4}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0808022B-9704-4150-8BFC-D3B6C7A25640}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E868B1FC-FDA7-4769-B050-5BF2503A6552}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FDF720B3-3595-49CC-902E-636FB545B866}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D00243A3-8AF8-403A-8C03-4281C387CE91}"/>
 </file>
</xml_diff>

<commit_message>
returns restock, both adjustment types, longer shipment codes
</commit_message>
<xml_diff>
--- a/Stock_Control/INRIPE_Stock_Entry_v1.xlsx
+++ b/Stock_Control/INRIPE_Stock_Entry_v1.xlsx
@@ -225,7 +225,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -306,6 +306,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00152947"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -396,7 +401,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -537,6 +542,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1056,14 +1064,14 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tblItems" displayName="tblItems" ref="B15:D47" headerRowCount="1">
-  <autoFilter ref="B15:D47"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tblItems" displayName="tblItems" ref="B15:D58" headerRowCount="1">
+  <autoFilter ref="B15:D58"/>
   <tableColumns count="3">
     <tableColumn id="2" name="Item Name"/>
     <tableColumn id="3" name="Item Code"/>
     <tableColumn id="4" name="Active"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
 </table>
 </file>
 
@@ -1649,7 +1657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB47"/>
+  <dimension ref="A1:AB58"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="55" min="1" max="1"/>
@@ -3172,6 +3180,193 @@
         </is>
       </c>
       <c r="D47" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="64" t="inlineStr">
+        <is>
+          <t>Watermelon</t>
+        </is>
+      </c>
+      <c r="C48" s="64" t="inlineStr">
+        <is>
+          <t>EG-FG-WTM-01-02-01-01</t>
+        </is>
+      </c>
+      <c r="D48" s="64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="64" t="inlineStr">
+        <is>
+          <t>Peach Sugary</t>
+        </is>
+      </c>
+      <c r="C49" s="64" t="inlineStr">
+        <is>
+          <t>EG-FG-PCH-01-02-01-01</t>
+        </is>
+      </c>
+      <c r="D49" s="64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="64" t="inlineStr">
+        <is>
+          <t>Apricot Amar</t>
+        </is>
+      </c>
+      <c r="C50" s="64" t="inlineStr">
+        <is>
+          <t>EG-FG-APR-01-02-01-01</t>
+        </is>
+      </c>
+      <c r="D50" s="64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="64" t="inlineStr">
+        <is>
+          <t>Peach Baladi</t>
+        </is>
+      </c>
+      <c r="C51" s="64" t="inlineStr">
+        <is>
+          <t>EG-FG-PCH-02-02-01-01</t>
+        </is>
+      </c>
+      <c r="D51" s="64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="64" t="inlineStr">
+        <is>
+          <t>Berries Omani</t>
+        </is>
+      </c>
+      <c r="C52" s="64" t="inlineStr">
+        <is>
+          <t>EG-FG-BER-01-02-01-01</t>
+        </is>
+      </c>
+      <c r="D52" s="64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="64" t="inlineStr">
+        <is>
+          <t>Grapes White</t>
+        </is>
+      </c>
+      <c r="C53" s="64" t="inlineStr">
+        <is>
+          <t>EG-FG-GRP-02-02-01-01</t>
+        </is>
+      </c>
+      <c r="D53" s="64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="64" t="inlineStr">
+        <is>
+          <t>Mango Timor Yemeni</t>
+        </is>
+      </c>
+      <c r="C54" s="64" t="inlineStr">
+        <is>
+          <t>EG-FG-MNG-16-01-01-01</t>
+        </is>
+      </c>
+      <c r="D54" s="64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="64" t="inlineStr">
+        <is>
+          <t>Plum Hollywood</t>
+        </is>
+      </c>
+      <c r="C55" s="64" t="inlineStr">
+        <is>
+          <t>EG-FG-PLM-01-02-01-01</t>
+        </is>
+      </c>
+      <c r="D55" s="64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="64" t="inlineStr">
+        <is>
+          <t>Golden Berry</t>
+        </is>
+      </c>
+      <c r="C56" s="64" t="inlineStr">
+        <is>
+          <t>EG-FG-GLD-01-02-01-01</t>
+        </is>
+      </c>
+      <c r="D56" s="64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="64" t="inlineStr">
+        <is>
+          <t>Bashmala</t>
+        </is>
+      </c>
+      <c r="C57" s="64" t="inlineStr">
+        <is>
+          <t>EG-FG-BSH-01-02-01-01</t>
+        </is>
+      </c>
+      <c r="D57" s="64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="64" t="inlineStr">
+        <is>
+          <t>Apple Baladi</t>
+        </is>
+      </c>
+      <c r="C58" s="64" t="inlineStr">
+        <is>
+          <t>EG-FG-APL-01-02-01-01</t>
+        </is>
+      </c>
+      <c r="D58" s="64" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4048,13 +4243,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B49B2771-1988-4B3E-A8BC-F5BBF35B9DDD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E851381-A0E2-40AA-A3AF-9A240AA726B1}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1AC40BED-4D94-43DF-AE3B-59A12FE7D057}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7BAD26A-5F61-4C15-9A21-64B892FD2FD8}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B35D5810-CB0B-423C-AABA-44927AEB8D16}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C1512BA-E2FD-41F7-95A2-271EF61283A5}"/>
 </file>
</xml_diff>